<commit_message>
feat(image-system): HISSA B — Excel image column in bulk import
- bulk_import_service: read optional image column from xlsx/csv rows;
  _find_library_image() does topic-scoped match first then global (case-
  insensitive, trimmed); on match copies library file to uploads/ and sets
  image_path; unknown name adds warning without skipping the question;
  column absent -> silent no-op (backward compat with old templates)
- bulk_upload_template.xlsx: image column added (col 13)
- 7 new tests in test_bulk_import_image.py (482 total); ruff clean
</commit_message>
<xml_diff>
--- a/static/bulk_upload_template.xlsx
+++ b/static/bulk_upload_template.xlsx
@@ -458,7 +458,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L5"/>
+  <dimension ref="A1:M5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -536,6 +536,11 @@
           <t>is_urdu</t>
         </is>
       </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>image</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -596,6 +601,7 @@
           <t>no</t>
         </is>
       </c>
+      <c r="M2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -749,9 +755,7 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr"/>
-    </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
feat: answer_lines column bulk Excel import mein add kiya
- bulk_import_service: answer_lines parse karo (valid: 0,2,3,4,6,8; invalid/blank = NULL + warning)
- questions_repository.insert: answer_lines column INSERT mein add kiya
- bulk_upload_template.xlsx: answer_lines column (green, optional) add kiya
- 11 nayi tests: valid values, zero, blank, invalid int, non-numeric, backward compat, parametrize
</commit_message>
<xml_diff>
--- a/static/bulk_upload_template.xlsx
+++ b/static/bulk_upload_template.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -29,8 +29,11 @@
       <b val="1"/>
       <color rgb="00FFFFFF"/>
     </font>
+    <font>
+      <b val="1"/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -47,6 +50,12 @@
         <fgColor rgb="003B7DC8"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C6EFCE"/>
+        <bgColor rgb="00C6EFCE"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -60,12 +69,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -433,7 +445,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U4"/>
+  <dimension ref="A1:V4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -457,6 +469,7 @@
     <col width="20" customWidth="1" min="19" max="19"/>
     <col width="14" customWidth="1" min="20" max="20"/>
     <col width="12" customWidth="1" min="21" max="21"/>
+    <col width="14" customWidth="1" min="22" max="22"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -565,6 +578,11 @@
           <t>status</t>
         </is>
       </c>
+      <c r="V1" s="3" t="inlineStr">
+        <is>
+          <t>answer_lines</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -625,7 +643,6 @@
           <t>no</t>
         </is>
       </c>
-      <c r="M2" t="inlineStr"/>
       <c r="N2" t="inlineStr">
         <is>
           <t>REMEMBER</t>
@@ -679,11 +696,6 @@
           <t>Science</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr"/>
-      <c r="E3" t="inlineStr"/>
-      <c r="F3" t="inlineStr"/>
-      <c r="G3" t="inlineStr"/>
-      <c r="H3" t="inlineStr"/>
       <c r="I3" t="n">
         <v>2</v>
       </c>
@@ -702,7 +714,6 @@
           <t>no</t>
         </is>
       </c>
-      <c r="M3" t="inlineStr"/>
       <c r="N3" t="inlineStr">
         <is>
           <t>UNDERSTAND</t>
@@ -718,14 +729,11 @@
           <t>water cycle, evaporation</t>
         </is>
       </c>
-      <c r="Q3" t="inlineStr"/>
-      <c r="R3" t="inlineStr"/>
       <c r="S3" t="inlineStr">
         <is>
           <t>NCERT Science 6</t>
         </is>
       </c>
-      <c r="T3" t="inlineStr"/>
       <c r="U3" t="inlineStr">
         <is>
           <t>published</t>
@@ -748,10 +756,6 @@
           <t>Science</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr"/>
-      <c r="E4" t="inlineStr"/>
-      <c r="F4" t="inlineStr"/>
-      <c r="G4" t="inlineStr"/>
       <c r="H4" t="inlineStr">
         <is>
           <t>true</t>
@@ -765,21 +769,11 @@
           <t>5</t>
         </is>
       </c>
-      <c r="K4" t="inlineStr"/>
       <c r="L4" t="inlineStr">
         <is>
           <t>no</t>
         </is>
       </c>
-      <c r="M4" t="inlineStr"/>
-      <c r="N4" t="inlineStr"/>
-      <c r="O4" t="inlineStr"/>
-      <c r="P4" t="inlineStr"/>
-      <c r="Q4" t="inlineStr"/>
-      <c r="R4" t="inlineStr"/>
-      <c r="S4" t="inlineStr"/>
-      <c r="T4" t="inlineStr"/>
-      <c r="U4" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
feat(slo): Marhala 2 Hissa A — Excel SLO tagging (bulk-upload + bulk-assign)
KAAM A — questions ko SLO se Excel se jodo (manual picker nahi):
- bulk question upload: naya optional slo_code column (comma-separated =
  kai SLO); ghalat code skip+warning, question phir bhi import
- purane questions: GET /api/questions/slo-export (question_id + current
  slo_code) + POST /api/slo/assign-import (id se match, replace-set)
- question_id column protection: import par saaf error (khali/unknown id),
  Excel cell-comment warning — over-engineer nahi
- shared resolve_slo_codes (case/space-insensitive), slo.html bulk-assign UI
- tests: +17 (730 total). Duplicate-on-reupload behavior documented+tested
  (bulk import upsert nahi karta — purane ke liye assign, re-upload nahi)

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/static/bulk_upload_template.xlsx
+++ b/static/bulk_upload_template.xlsx
@@ -445,7 +445,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V4"/>
+  <dimension ref="A1:W4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -583,6 +583,11 @@
           <t>answer_lines</t>
         </is>
       </c>
+      <c r="W1" t="inlineStr">
+        <is>
+          <t>slo_code</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -679,6 +684,7 @@
           <t>published</t>
         </is>
       </c>
+      <c r="W2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -739,6 +745,11 @@
           <t>published</t>
         </is>
       </c>
+      <c r="W3" t="inlineStr">
+        <is>
+          <t>SCI-01, SCI-02</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -774,6 +785,7 @@
           <t>no</t>
         </is>
       </c>
+      <c r="W4" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>